<commit_message>
Normalisation of experimental factors part 2
Added experimental factor levels. This is used to capture details for each factor level. It links to experimental factors on the expeFactorId column, and introduces a readonly expeFactorLevelId value which is a unique identifier across studies by concatenating the factor id with the level code.
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98C83358-2032-4458-95BE-E8D2655F1635}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A8704DE-36BD-45DC-94E5-6E0416144695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1000" uniqueCount="685">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="691">
   <si>
     <t>README</t>
   </si>
@@ -2292,6 +2292,24 @@
   <si>
     <t>N</t>
   </si>
+  <si>
+    <t>expeFactorLevelId</t>
+  </si>
+  <si>
+    <t>expeFactorLevel</t>
+  </si>
+  <si>
+    <t>expeFactorLevelAccession</t>
+  </si>
+  <si>
+    <t>expeFactorLevelDesc</t>
+  </si>
+  <si>
+    <t>S1-N</t>
+  </si>
+  <si>
+    <t>N1</t>
+  </si>
 </sst>
 </file>
 
@@ -2300,7 +2318,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="26" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2486,6 +2504,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006AB9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2545,7 +2569,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="68">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2714,6 +2738,7 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5338,6 +5363,22 @@
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:G2" insertRow="1" totalsRowShown="0" dataDxfId="32">
+  <autoFilter ref="A1:G2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="39"/>
+    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="37"/>
+    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="36"/>
+    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="35"/>
+    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="34"/>
+    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="33"/>
+  </tableColumns>
+  <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="24">
   <autoFilter ref="A1:G2" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}"/>
   <tableColumns count="7">
@@ -5353,7 +5394,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:Q2" insertRow="1" totalsRowShown="0" dataDxfId="5">
   <autoFilter ref="A1:Q2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
   <tableColumns count="17">
@@ -5379,7 +5420,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C3" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}"/>
   <tableColumns count="3">
@@ -5511,6 +5552,22 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="13" xr:uid="{C9BF05A2-1ABB-4D33-BC15-C5E51AF45999}" name="experimentFactorLevel" displayName="experimentFactorLevel" ref="A1:E2" totalsRowShown="0">
+  <autoFilter ref="A1:E2" xr:uid="{C9BF05A2-1ABB-4D33-BC15-C5E51AF45999}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{87ACD6F9-EF3B-4A5E-B872-92E772B18A0D}" name="expeFactorId"/>
+    <tableColumn id="2" xr3:uid="{684FB454-4CC5-45F7-9C3C-B04475EADF64}" name="expeFactorLevelId">
+      <calculatedColumnFormula>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevel])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="3" xr3:uid="{1C4A38F3-CA10-4B27-8557-5CEB94A37762}" name="expeFactorLevel"/>
+    <tableColumn id="4" xr3:uid="{8AD64F88-1111-477C-8058-D8790CFA7C77}" name="expeFactorLevelAccession"/>
+    <tableColumn id="5" xr3:uid="{925EFD52-D576-4B2F-BE3D-7FEE62D537D8}" name="expeFactorLevelDesc"/>
+  </tableColumns>
+  <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:F2" insertRow="1" totalsRowShown="0" dataDxfId="40">
   <autoFilter ref="A1:F2" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}"/>
   <tableColumns count="6">
@@ -5520,22 +5577,6 @@
     <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="43"/>
     <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="42"/>
     <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="41"/>
-  </tableColumns>
-  <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:G2" insertRow="1" totalsRowShown="0" dataDxfId="32">
-  <autoFilter ref="A1:G2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="33"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -24321,9 +24362,57 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D0E16F6-2188-4422-AF91-E595A36EE21A}">
-  <dimension ref="A1"/>
+  <sheetPr>
+    <tabColor theme="5"/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="14.07421875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.765625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.07421875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.53515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.07421875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A1" t="s">
+        <v>681</v>
+      </c>
+      <c r="B1" s="68" t="s">
+        <v>685</v>
+      </c>
+      <c r="C1" t="s">
+        <v>686</v>
+      </c>
+      <c r="D1" t="s">
+        <v>687</v>
+      </c>
+      <c r="E1" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.4">
+      <c r="A2" t="s">
+        <v>689</v>
+      </c>
+      <c r="B2" t="str">
+        <f>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevel])</f>
+        <v>S1-N-N1</v>
+      </c>
+      <c r="C2" s="63" t="s">
+        <v>690</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{BB15239E-DF5D-4524-AED3-F9F9639D5B2D}">
+      <formula1>INDIRECT("experimentalFactor[expeFactorId]")</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Standardising observed variable  column names
Standardised accession names as various forms were used (Acc, AccNumber, Accession) to just use accession - accession and number are slightly tautological:
variableAccession, traitNameAccession,  traitCharacteristicAccession, methodAccession, scaleAccession
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A8704DE-36BD-45DC-94E5-6E0416144695}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDA4427-A835-4119-9894-C17474B04E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="691">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="697">
   <si>
     <t>README</t>
   </si>
@@ -2296,9 +2296,6 @@
     <t>expeFactorLevelId</t>
   </si>
   <si>
-    <t>expeFactorLevel</t>
-  </si>
-  <si>
     <t>expeFactorLevelAccession</t>
   </si>
   <si>
@@ -2309,6 +2306,27 @@
   </si>
   <si>
     <t>N1</t>
+  </si>
+  <si>
+    <t>expeFactorLevelCode</t>
+  </si>
+  <si>
+    <t>variableAccession</t>
+  </si>
+  <si>
+    <t>traitEntityAccession</t>
+  </si>
+  <si>
+    <t>traitCharacteristicAccession</t>
+  </si>
+  <si>
+    <t>traitAccession</t>
+  </si>
+  <si>
+    <t>methodAccession</t>
+  </si>
+  <si>
+    <t>scaleAccession</t>
   </si>
 </sst>
 </file>
@@ -2747,6 +2765,26 @@
   <dxfs count="134">
     <dxf>
       <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <strike val="0"/>
@@ -3062,26 +3100,6 @@
         <scheme val="none"/>
       </font>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Arial"/>
-        <family val="2"/>
-        <charset val="1"/>
-        <scheme val="none"/>
-      </font>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -5395,33 +5413,33 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:Q2" insertRow="1" totalsRowShown="0" dataDxfId="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:Q2" insertRow="1" totalsRowShown="0" dataDxfId="6">
   <autoFilter ref="A1:Q2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
   <tableColumns count="17">
     <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="22"/>
     <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="21"/>
     <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccNumber" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="19"/>
     <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="17"/>
-    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccessionNumber" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccessionNumber" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccNumber" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="12"/>
-    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccNumber" dataDxfId="11"/>
-    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="10"/>
-    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="9"/>
-    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="8"/>
-    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccNumber" dataDxfId="7"/>
-    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="timeScale" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="0"/>
+    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="16"/>
+    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="15"/>
+    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="14"/>
+    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="13"/>
+    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="11"/>
+    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="10"/>
+    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="9"/>
+    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="timeScale" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="4">
   <autoFilter ref="A1:C3" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5E761B2A-3F92-4181-AF5D-F423F0564A09}" name="envParam"/>
@@ -5437,7 +5455,7 @@
   <autoFilter ref="A1:T3" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}"/>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="114"/>
-    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="parentStudyId" dataDxfId="4"/>
+    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="parentStudyId" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="113"/>
     <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="112"/>
     <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="111"/>
@@ -5539,13 +5557,13 @@
   <autoFilter ref="A1:F2" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="1"/>
-    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="2">
+    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="3">
       <calculatedColumnFormula>CONCATENATE(experimentalFactor[studyId],"-",experimentalFactor[expeFactorCode])</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="49"/>
     <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5557,9 +5575,9 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{87ACD6F9-EF3B-4A5E-B872-92E772B18A0D}" name="expeFactorId"/>
     <tableColumn id="2" xr3:uid="{684FB454-4CC5-45F7-9C3C-B04475EADF64}" name="expeFactorLevelId">
-      <calculatedColumnFormula>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevel])</calculatedColumnFormula>
+      <calculatedColumnFormula>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevelCode])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{1C4A38F3-CA10-4B27-8557-5CEB94A37762}" name="expeFactorLevel"/>
+    <tableColumn id="3" xr3:uid="{1C4A38F3-CA10-4B27-8557-5CEB94A37762}" name="expeFactorLevelCode"/>
     <tableColumn id="4" xr3:uid="{8AD64F88-1111-477C-8058-D8790CFA7C77}" name="expeFactorLevelAccession"/>
     <tableColumn id="5" xr3:uid="{925EFD52-D576-4B2F-BE3D-7FEE62D537D8}" name="expeFactorLevelDesc"/>
   </tableColumns>
@@ -13584,8 +13602,8 @@
     <col min="2" max="2" width="11.4609375" customWidth="1"/>
     <col min="3" max="3" width="14.84375" customWidth="1"/>
     <col min="4" max="4" width="19.69140625" customWidth="1"/>
-    <col min="5" max="5" width="11.15234375" customWidth="1"/>
-    <col min="6" max="6" width="10.921875" customWidth="1"/>
+    <col min="5" max="5" width="14.765625" customWidth="1"/>
+    <col min="6" max="6" width="13.69140625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.15234375" customWidth="1"/>
     <col min="8" max="8" width="17.921875" customWidth="1"/>
     <col min="9" max="9" width="33.15234375" customWidth="1"/>
@@ -13612,7 +13630,7 @@
         <v>389</v>
       </c>
       <c r="D1" s="59" t="s">
-        <v>390</v>
+        <v>691</v>
       </c>
       <c r="E1" s="57" t="s">
         <v>391</v>
@@ -13621,22 +13639,22 @@
         <v>392</v>
       </c>
       <c r="G1" s="59" t="s">
-        <v>393</v>
+        <v>692</v>
       </c>
       <c r="H1" s="59" t="s">
         <v>394</v>
       </c>
       <c r="I1" s="59" t="s">
-        <v>395</v>
+        <v>693</v>
       </c>
       <c r="J1" s="59" t="s">
-        <v>396</v>
+        <v>694</v>
       </c>
       <c r="K1" s="57" t="s">
         <v>397</v>
       </c>
       <c r="L1" s="59" t="s">
-        <v>398</v>
+        <v>695</v>
       </c>
       <c r="M1" s="58" t="s">
         <v>399</v>
@@ -13648,7 +13666,7 @@
         <v>401</v>
       </c>
       <c r="P1" s="59" t="s">
-        <v>402</v>
+        <v>696</v>
       </c>
       <c r="Q1" s="59" t="s">
         <v>403</v>
@@ -24370,8 +24388,8 @@
   <cols>
     <col min="1" max="1" width="14.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.765625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.07421875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.53515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="21.4609375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.53515625" customWidth="1"/>
     <col min="5" max="5" width="21.07421875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -24382,26 +24400,26 @@
       <c r="B1" s="68" t="s">
         <v>685</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="63" t="s">
+        <v>690</v>
+      </c>
+      <c r="D1" t="s">
         <v>686</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>687</v>
-      </c>
-      <c r="E1" t="s">
-        <v>688</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>688</v>
+      </c>
+      <c r="B2" t="str">
+        <f>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevelCode])</f>
+        <v>S1-N-N1</v>
+      </c>
+      <c r="C2" s="63" t="s">
         <v>689</v>
-      </c>
-      <c r="B2" t="str">
-        <f>CONCATENATE(experimentFactorLevel[expeFactorId],"-",experimentFactorLevel[expeFactorLevel])</f>
-        <v>S1-N-N1</v>
-      </c>
-      <c r="C2" s="63" t="s">
-        <v>690</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new participant fields to observed variable
The participant and participantRole (with accompanying accession fields are designed to capture biological, chemical or other entities that are central to interpretation of a variable but not full captured in the trait, for example, it allows a disease trait variable to capture the pathoogen and its role with respect to the entity (e.g. pathogen of)
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DDA4427-A835-4119-9894-C17474B04E1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E08564F4-4A13-4326-8E07-228211CF19C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="1725" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="15" windowWidth="29040" windowHeight="16440" tabRatio="891" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1007" uniqueCount="697">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="701">
   <si>
     <t>README</t>
   </si>
@@ -2327,6 +2327,18 @@
   </si>
   <si>
     <t>scaleAccession</t>
+  </si>
+  <si>
+    <t>participant</t>
+  </si>
+  <si>
+    <t>participantAccession</t>
+  </si>
+  <si>
+    <t>participantRole</t>
+  </si>
+  <si>
+    <t>participantRoleAccession</t>
   </si>
 </sst>
 </file>
@@ -2762,7 +2774,87 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="134">
+  <dxfs count="138">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -5341,15 +5433,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="MiappeStyle" pivot="0" count="9" xr9:uid="{59C54380-D204-4007-9CC6-0890CCDEE3C9}">
-      <tableStyleElement type="wholeTable" dxfId="133"/>
-      <tableStyleElement type="headerRow" dxfId="132"/>
-      <tableStyleElement type="totalRow" dxfId="131"/>
-      <tableStyleElement type="firstColumn" dxfId="130"/>
-      <tableStyleElement type="lastColumn" dxfId="129"/>
-      <tableStyleElement type="firstRowStripe" dxfId="128"/>
-      <tableStyleElement type="secondRowStripe" dxfId="127"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="126"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="125"/>
+      <tableStyleElement type="wholeTable" dxfId="137"/>
+      <tableStyleElement type="headerRow" dxfId="136"/>
+      <tableStyleElement type="totalRow" dxfId="135"/>
+      <tableStyleElement type="firstColumn" dxfId="134"/>
+      <tableStyleElement type="lastColumn" dxfId="133"/>
+      <tableStyleElement type="firstRowStripe" dxfId="132"/>
+      <tableStyleElement type="secondRowStripe" dxfId="131"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="130"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="129"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -5364,82 +5456,86 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="115" dataDxfId="116">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="119" dataDxfId="120">
   <autoFilter ref="A1:H2" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="124"/>
-    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="123"/>
-    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="122"/>
-    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="121"/>
-    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="120"/>
-    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="119"/>
-    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="118"/>
-    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="117"/>
+    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="128"/>
+    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="127"/>
+    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="126"/>
+    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="125"/>
+    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="124"/>
+    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="123"/>
+    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="122"/>
+    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="121"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:G2" insertRow="1" totalsRowShown="0" dataDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:G2" insertRow="1" totalsRowShown="0" dataDxfId="36">
   <autoFilter ref="A1:G2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="39"/>
-    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="38"/>
-    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="37"/>
-    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="36"/>
-    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="35"/>
-    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="34"/>
-    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="43"/>
+    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="42"/>
+    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="41"/>
+    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="40"/>
+    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="39"/>
+    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="38"/>
+    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="37"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="23" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="28">
   <autoFilter ref="A1:G2" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="31"/>
-    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="30"/>
-    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="29"/>
-    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="28"/>
-    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="27"/>
-    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="26"/>
-    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="35"/>
+    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="34"/>
+    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="33"/>
+    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="31"/>
+    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="30"/>
+    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="29"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:Q2" insertRow="1" totalsRowShown="0" dataDxfId="6">
-  <autoFilter ref="A1:Q2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
-  <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="19"/>
-    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="18"/>
-    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="0"/>
-    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="17"/>
-    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="16"/>
-    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="15"/>
-    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="14"/>
-    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="13"/>
-    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="12"/>
-    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="10"/>
-    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="9"/>
-    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="8"/>
-    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="timeScale" dataDxfId="7"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:U2" insertRow="1" totalsRowShown="0" dataDxfId="10">
+  <autoFilter ref="A1:U2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
+  <tableColumns count="21">
+    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="25"/>
+    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="21"/>
+    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="20"/>
+    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="19"/>
+    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="18"/>
+    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="17"/>
+    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="16"/>
+    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="15"/>
+    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="14"/>
+    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="13"/>
+    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="12"/>
+    <tableColumn id="19" xr3:uid="{EE91A801-8376-4314-ADFB-6E32C3AE8AE4}" name="timeScale" dataDxfId="3"/>
+    <tableColumn id="22" xr3:uid="{A52D8785-E3B2-4548-AA8A-0964285F0DB9}" name="participant" dataDxfId="0"/>
+    <tableColumn id="21" xr3:uid="{CA21FA4C-5A61-4852-9BA7-6FDDF22D4ADC}" name="participantAccession" dataDxfId="1"/>
+    <tableColumn id="20" xr3:uid="{3DF54E16-A553-4C7E-9762-C6517F5AD994}" name="participantRole" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="participantRoleAccession" dataDxfId="11"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="4">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="8">
   <autoFilter ref="A1:C3" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5E761B2A-3F92-4181-AF5D-F423F0564A09}" name="envParam"/>
@@ -5451,119 +5547,119 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="95">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="99">
   <autoFilter ref="A1:T3" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="114"/>
-    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="parentStudyId" dataDxfId="5"/>
-    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="113"/>
-    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="112"/>
-    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="111"/>
-    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="110"/>
-    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="109"/>
-    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="108"/>
-    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="107"/>
-    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="106"/>
-    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="105"/>
-    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="104"/>
-    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="103"/>
-    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="102"/>
-    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="101"/>
-    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="100"/>
-    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="99"/>
-    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="98"/>
-    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="97"/>
-    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="96"/>
+    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="118"/>
+    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="parentStudyId" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="117"/>
+    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="116"/>
+    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="115"/>
+    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="114"/>
+    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="113"/>
+    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="112"/>
+    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="111"/>
+    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="110"/>
+    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="109"/>
+    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="108"/>
+    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="107"/>
+    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="106"/>
+    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="105"/>
+    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="104"/>
+    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="103"/>
+    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="102"/>
+    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="101"/>
+    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="100"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="87" dataDxfId="88">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="91" dataDxfId="92">
   <autoFilter ref="A1:F2" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="94"/>
-    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="93"/>
-    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="92"/>
-    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="91"/>
-    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="90"/>
-    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="89"/>
+    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="98"/>
+    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="97"/>
+    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="96"/>
+    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="95"/>
+    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="94"/>
+    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="93"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="81" dataDxfId="82">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="85" dataDxfId="86">
   <autoFilter ref="A1:D2" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="86"/>
-    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="85"/>
-    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="84"/>
-    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="83"/>
+    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="90"/>
+    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="89"/>
+    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="88"/>
+    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="87"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="55" dataDxfId="56">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="59" dataDxfId="60">
   <autoFilter ref="A1:X2" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="80"/>
-    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="79"/>
-    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="78"/>
-    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="77"/>
-    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="76"/>
-    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="75"/>
-    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="74"/>
-    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="73"/>
-    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="72"/>
-    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="71"/>
-    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="70"/>
-    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="69"/>
-    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="68"/>
-    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="67"/>
-    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="66"/>
-    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="65"/>
-    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="64"/>
-    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="63"/>
-    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="62"/>
-    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="61"/>
-    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="60"/>
-    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="59"/>
-    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="58"/>
-    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="57"/>
+    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="84"/>
+    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="83"/>
+    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="82"/>
+    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="81"/>
+    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="80"/>
+    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="79"/>
+    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="78"/>
+    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="77"/>
+    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="76"/>
+    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="75"/>
+    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="74"/>
+    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="73"/>
+    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="72"/>
+    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="71"/>
+    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="70"/>
+    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="69"/>
+    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="68"/>
+    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="67"/>
+    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="66"/>
+    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="65"/>
+    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="64"/>
+    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="63"/>
+    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="62"/>
+    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="61"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="51">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="55">
   <autoFilter ref="A1:C2" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="54"/>
-    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="53"/>
-    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="52"/>
+    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="58"/>
+    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="57"/>
+    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="56"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="47">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="51">
   <autoFilter ref="A1:F2" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="50"/>
-    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="54"/>
+    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="7">
       <calculatedColumnFormula>CONCATENATE(experimentalFactor[studyId],"-",experimentalFactor[expeFactorCode])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="49"/>
-    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="48"/>
-    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="53"/>
+    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="52"/>
+    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5586,15 +5682,15 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:F2" insertRow="1" totalsRowShown="0" dataDxfId="40">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:F2" insertRow="1" totalsRowShown="0" dataDxfId="44">
   <autoFilter ref="A1:F2" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="46"/>
-    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="45"/>
-    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="44"/>
-    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="43"/>
-    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="42"/>
-    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="41"/>
+    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="50"/>
+    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="49"/>
+    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="48"/>
+    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="47"/>
+    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="46"/>
+    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="45"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -13595,7 +13691,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:Q997"/>
+  <dimension ref="A1:U997"/>
   <sheetFormatPr defaultColWidth="14.53515625" defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="8.921875" customWidth="1"/>
@@ -13613,13 +13709,15 @@
     <col min="13" max="13" width="13.3046875" customWidth="1"/>
     <col min="14" max="14" width="12.15234375" customWidth="1"/>
     <col min="15" max="15" width="12.23046875" customWidth="1"/>
-    <col min="16" max="16" width="17.07421875" customWidth="1"/>
-    <col min="17" max="17" width="11.4609375" customWidth="1"/>
-    <col min="16379" max="16379" width="11.4609375" customWidth="1"/>
-    <col min="16380" max="16384" width="11.53515625" customWidth="1"/>
+    <col min="16" max="18" width="17.07421875" customWidth="1"/>
+    <col min="19" max="19" width="23.84375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.61328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="27.84375" bestFit="1" customWidth="1"/>
+    <col min="16383" max="16383" width="11.4609375" customWidth="1"/>
+    <col min="16384" max="16384" width="11.53515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="37" customFormat="1" ht="25.4" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:21" s="37" customFormat="1" ht="25.4" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A1" s="57" t="s">
         <v>66</v>
       </c>
@@ -13671,8 +13769,20 @@
       <c r="Q1" s="59" t="s">
         <v>403</v>
       </c>
-    </row>
-    <row r="2" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R1" s="59" t="s">
+        <v>697</v>
+      </c>
+      <c r="S1" s="59" t="s">
+        <v>698</v>
+      </c>
+      <c r="T1" s="59" t="s">
+        <v>699</v>
+      </c>
+      <c r="U1" s="59" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="55"/>
       <c r="B2" s="54"/>
       <c r="C2" s="55"/>
@@ -13690,8 +13800,12 @@
       <c r="O2" s="54"/>
       <c r="P2" s="54"/>
       <c r="Q2" s="54"/>
-    </row>
-    <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R2" s="54"/>
+      <c r="S2" s="54"/>
+      <c r="T2" s="54"/>
+      <c r="U2" s="54"/>
+    </row>
+    <row r="3" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" s="56"/>
       <c r="B3" s="56"/>
       <c r="C3" s="56"/>
@@ -13709,8 +13823,12 @@
       <c r="O3" s="56"/>
       <c r="P3" s="56"/>
       <c r="Q3" s="56"/>
-    </row>
-    <row r="4" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R3" s="56"/>
+      <c r="S3" s="56"/>
+      <c r="T3" s="56"/>
+      <c r="U3" s="56"/>
+    </row>
+    <row r="4" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A4" s="56"/>
       <c r="B4" s="56"/>
       <c r="C4" s="56"/>
@@ -13728,8 +13846,12 @@
       <c r="O4" s="56"/>
       <c r="P4" s="56"/>
       <c r="Q4" s="56"/>
-    </row>
-    <row r="5" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R4" s="56"/>
+      <c r="S4" s="56"/>
+      <c r="T4" s="56"/>
+      <c r="U4" s="56"/>
+    </row>
+    <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="56"/>
       <c r="B5" s="56"/>
       <c r="C5" s="56"/>
@@ -13747,8 +13869,12 @@
       <c r="O5" s="56"/>
       <c r="P5" s="56"/>
       <c r="Q5" s="56"/>
-    </row>
-    <row r="6" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R5" s="56"/>
+      <c r="S5" s="56"/>
+      <c r="T5" s="56"/>
+      <c r="U5" s="56"/>
+    </row>
+    <row r="6" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="56"/>
       <c r="B6" s="56"/>
       <c r="C6" s="56"/>
@@ -13766,8 +13892,12 @@
       <c r="O6" s="56"/>
       <c r="P6" s="56"/>
       <c r="Q6" s="56"/>
-    </row>
-    <row r="7" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R6" s="56"/>
+      <c r="S6" s="56"/>
+      <c r="T6" s="56"/>
+      <c r="U6" s="56"/>
+    </row>
+    <row r="7" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A7" s="56"/>
       <c r="B7" s="56"/>
       <c r="C7" s="56"/>
@@ -13785,8 +13915,12 @@
       <c r="O7" s="56"/>
       <c r="P7" s="56"/>
       <c r="Q7" s="56"/>
-    </row>
-    <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="R7" s="56"/>
+      <c r="S7" s="56"/>
+      <c r="T7" s="56"/>
+      <c r="U7" s="56"/>
+    </row>
+    <row r="8" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A8" s="56"/>
       <c r="B8" s="56"/>
       <c r="C8" s="56"/>
@@ -13804,15 +13938,19 @@
       <c r="O8" s="56"/>
       <c r="P8" s="56"/>
       <c r="Q8" s="56"/>
-    </row>
-    <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="10" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="11" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="12" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="13" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="14" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="15" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="16" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+      <c r="R8" s="56"/>
+      <c r="S8" s="56"/>
+      <c r="T8" s="56"/>
+      <c r="U8" s="56"/>
+    </row>
+    <row r="9" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="10" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="11" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="12" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="13" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="14" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="15" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
+    <row r="16" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>
     <row r="19" ht="15.75" customHeight="1" x14ac:dyDescent="0.4"/>

</xml_diff>

<commit_message>
renamed parentStudyId to sourceStudyId
Provides a better description
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B29B008-B3ED-42A1-BE9D-B98EF601CD0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8203694-3FCC-49FE-B693-04E767C996D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -2186,9 +2186,6 @@
   </si>
   <si>
     <t>S2</t>
-  </si>
-  <si>
-    <t>parentStudyId</t>
   </si>
   <si>
     <t>envParamAccession</t>
@@ -2343,6 +2340,9 @@
   <si>
     <t>S1-N-N1</t>
   </si>
+  <si>
+    <t>sourceStudyId</t>
+  </si>
 </sst>
 </file>
 
@@ -2351,7 +2351,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2543,6 +2543,14 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF247A00"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -2602,7 +2610,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -2765,6 +2773,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -5567,7 +5578,7 @@
   <autoFilter ref="A1:T3" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}"/>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="96"/>
-    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="parentStudyId" dataDxfId="95"/>
+    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="sourceStudyId" dataDxfId="95"/>
     <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="94"/>
     <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="93"/>
     <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="92"/>
@@ -5952,7 +5963,7 @@
     </row>
     <row r="3" spans="1:20 16374:16384" s="9" customFormat="1" ht="98.45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>683</v>
+        <v>682</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -10243,7 +10254,7 @@
         <v>299</v>
       </c>
       <c r="C1" s="51" t="s">
-        <v>685</v>
+        <v>684</v>
       </c>
       <c r="D1" s="52" t="s">
         <v>300</v>
@@ -10269,7 +10280,7 @@
       <c r="A2" s="30"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13" t="s">
-        <v>701</v>
+        <v>700</v>
       </c>
       <c r="D2" s="13"/>
       <c r="E2" s="30"/>
@@ -13754,7 +13765,7 @@
         <v>389</v>
       </c>
       <c r="D1" s="56" t="s">
-        <v>691</v>
+        <v>690</v>
       </c>
       <c r="E1" s="54" t="s">
         <v>391</v>
@@ -13763,22 +13774,22 @@
         <v>392</v>
       </c>
       <c r="G1" s="56" t="s">
-        <v>692</v>
+        <v>691</v>
       </c>
       <c r="H1" s="56" t="s">
         <v>394</v>
       </c>
       <c r="I1" s="56" t="s">
+        <v>692</v>
+      </c>
+      <c r="J1" s="56" t="s">
         <v>693</v>
-      </c>
-      <c r="J1" s="56" t="s">
-        <v>694</v>
       </c>
       <c r="K1" s="54" t="s">
         <v>397</v>
       </c>
       <c r="L1" s="56" t="s">
-        <v>695</v>
+        <v>694</v>
       </c>
       <c r="M1" s="55" t="s">
         <v>399</v>
@@ -13790,22 +13801,22 @@
         <v>401</v>
       </c>
       <c r="P1" s="56" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
       <c r="Q1" s="56" t="s">
         <v>403</v>
       </c>
       <c r="R1" s="56" t="s">
+        <v>696</v>
+      </c>
+      <c r="S1" s="56" t="s">
         <v>697</v>
       </c>
-      <c r="S1" s="56" t="s">
+      <c r="T1" s="56" t="s">
         <v>698</v>
       </c>
-      <c r="T1" s="56" t="s">
+      <c r="U1" s="56" t="s">
         <v>699</v>
-      </c>
-      <c r="U1" s="56" t="s">
-        <v>700</v>
       </c>
     </row>
     <row r="2" spans="1:21" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -14989,29 +15000,29 @@
         <v>270</v>
       </c>
       <c r="B1" s="60" t="s">
+        <v>673</v>
+      </c>
+      <c r="C1" s="60" t="s">
         <v>674</v>
-      </c>
-      <c r="C1" s="60" t="s">
-        <v>675</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="61" t="s">
+        <v>675</v>
+      </c>
+      <c r="B2" s="62" t="s">
         <v>676</v>
       </c>
-      <c r="B2" s="62" t="s">
+      <c r="C2" t="s">
         <v>677</v>
-      </c>
-      <c r="C2" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>678</v>
+      </c>
+      <c r="B3" s="62" t="s">
         <v>679</v>
-      </c>
-      <c r="B3" s="62" t="s">
-        <v>680</v>
       </c>
     </row>
   </sheetData>
@@ -19568,8 +19579,8 @@
       <c r="A1" s="52" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="52" t="s">
-        <v>673</v>
+      <c r="B1" s="66" t="s">
+        <v>701</v>
       </c>
       <c r="C1" s="52" t="s">
         <v>67</v>
@@ -24327,10 +24338,10 @@
         <v>66</v>
       </c>
       <c r="B1" s="52" t="s">
-        <v>682</v>
+        <v>681</v>
       </c>
       <c r="C1" s="64" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="D1" s="52" t="s">
         <v>282</v>
@@ -24356,7 +24367,7 @@
         <v>671</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>684</v>
+        <v>683</v>
       </c>
       <c r="C2" s="30" t="str">
         <f>CONCATENATE(experimentalFactor[studyId],"-",experimentalFactor[expeFactorCode])</f>
@@ -24559,31 +24570,31 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>681</v>
+        <v>680</v>
       </c>
       <c r="B1" s="65" t="s">
+        <v>684</v>
+      </c>
+      <c r="C1" s="60" t="s">
+        <v>689</v>
+      </c>
+      <c r="D1" t="s">
         <v>685</v>
       </c>
-      <c r="C1" s="60" t="s">
-        <v>690</v>
-      </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>686</v>
-      </c>
-      <c r="E1" t="s">
-        <v>687</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>688</v>
+        <v>687</v>
       </c>
       <c r="B2" t="str">
         <f>CONCATENATE(experimentalFactorLevel[expeFactorId],"-",experimentalFactorLevel[expeFactorLevelCode])</f>
         <v>S1-N-N1</v>
       </c>
       <c r="C2" s="60" t="s">
-        <v>689</v>
+        <v>688</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added sourceObsUnitId to Observation Unit
Enables explicit linkage of an observation unit in one study to an observation unit in another study
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8203694-3FCC-49FE-B693-04E767C996D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D6E3BB-274C-4AD8-8440-6EF7D8E42893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1013" uniqueCount="702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="703">
   <si>
     <t>README</t>
   </si>
@@ -2342,6 +2342,9 @@
   </si>
   <si>
     <t>sourceStudyId</t>
+  </si>
+  <si>
+    <t>sourceObsUnitId</t>
   </si>
 </sst>
 </file>
@@ -2781,7 +2784,27 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="139">
+  <dxfs count="140">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -5460,15 +5483,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="MiappeStyle" pivot="0" count="9" xr9:uid="{59C54380-D204-4007-9CC6-0890CCDEE3C9}">
-      <tableStyleElement type="wholeTable" dxfId="138"/>
-      <tableStyleElement type="headerRow" dxfId="137"/>
-      <tableStyleElement type="totalRow" dxfId="136"/>
-      <tableStyleElement type="firstColumn" dxfId="135"/>
-      <tableStyleElement type="lastColumn" dxfId="134"/>
-      <tableStyleElement type="firstRowStripe" dxfId="133"/>
-      <tableStyleElement type="secondRowStripe" dxfId="132"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="131"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="130"/>
+      <tableStyleElement type="wholeTable" dxfId="139"/>
+      <tableStyleElement type="headerRow" dxfId="138"/>
+      <tableStyleElement type="totalRow" dxfId="137"/>
+      <tableStyleElement type="firstColumn" dxfId="136"/>
+      <tableStyleElement type="lastColumn" dxfId="135"/>
+      <tableStyleElement type="firstRowStripe" dxfId="134"/>
+      <tableStyleElement type="secondRowStripe" dxfId="133"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="132"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="131"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -5483,86 +5506,87 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="107" dataDxfId="106">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
   <autoFilter ref="A1:H2" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="105"/>
-    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="104"/>
-    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="103"/>
-    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="102"/>
-    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="101"/>
-    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="100"/>
-    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="99"/>
-    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="98"/>
+    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="106"/>
+    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="105"/>
+    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="104"/>
+    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="103"/>
+    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="102"/>
+    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="101"/>
+    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="100"/>
+    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="99"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:G2" insertRow="1" totalsRowShown="0" dataDxfId="18">
-  <autoFilter ref="A1:G2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
-  <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="17"/>
-    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="16"/>
-    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="15"/>
-    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="11"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:H2" insertRow="1" totalsRowShown="0" dataDxfId="19">
+  <autoFilter ref="A1:H2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{F4D9572F-C227-480C-812D-9943C387240C}" name="sourceObsUnitId" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="15"/>
+    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="14"/>
+    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="13"/>
+    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="12"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="10" dataDxfId="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
   <autoFilter ref="A1:G2" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="9"/>
+    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="8"/>
+    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="7"/>
+    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="3"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:U2" insertRow="1" totalsRowShown="0" dataDxfId="129">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:U2" insertRow="1" totalsRowShown="0" dataDxfId="130">
   <autoFilter ref="A1:U2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="128"/>
-    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="127"/>
-    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="126"/>
-    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="125"/>
-    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="124"/>
-    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="123"/>
-    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="122"/>
-    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="121"/>
-    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="120"/>
-    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="119"/>
-    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="118"/>
-    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="117"/>
-    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="116"/>
-    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="115"/>
-    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="114"/>
-    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="113"/>
-    <tableColumn id="19" xr3:uid="{EE91A801-8376-4314-ADFB-6E32C3AE8AE4}" name="timeScale" dataDxfId="112"/>
-    <tableColumn id="22" xr3:uid="{A52D8785-E3B2-4548-AA8A-0964285F0DB9}" name="participant" dataDxfId="111"/>
-    <tableColumn id="21" xr3:uid="{CA21FA4C-5A61-4852-9BA7-6FDDF22D4ADC}" name="participantAccession" dataDxfId="110"/>
-    <tableColumn id="20" xr3:uid="{3DF54E16-A553-4C7E-9762-C6517F5AD994}" name="participantRole" dataDxfId="109"/>
-    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="participantRoleAccession" dataDxfId="108"/>
+    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="129"/>
+    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="128"/>
+    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="127"/>
+    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="126"/>
+    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="125"/>
+    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="124"/>
+    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="123"/>
+    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="122"/>
+    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="121"/>
+    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="120"/>
+    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="119"/>
+    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="118"/>
+    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="117"/>
+    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="116"/>
+    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="115"/>
+    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="114"/>
+    <tableColumn id="19" xr3:uid="{EE91A801-8376-4314-ADFB-6E32C3AE8AE4}" name="timeScale" dataDxfId="113"/>
+    <tableColumn id="22" xr3:uid="{A52D8785-E3B2-4548-AA8A-0964285F0DB9}" name="participant" dataDxfId="112"/>
+    <tableColumn id="21" xr3:uid="{CA21FA4C-5A61-4852-9BA7-6FDDF22D4ADC}" name="participantAccession" dataDxfId="111"/>
+    <tableColumn id="20" xr3:uid="{3DF54E16-A553-4C7E-9762-C6517F5AD994}" name="participantRole" dataDxfId="110"/>
+    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="participantRoleAccession" dataDxfId="109"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="2">
   <autoFilter ref="A1:C3" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5E761B2A-3F92-4181-AF5D-F423F0564A09}" name="envParam"/>
@@ -5574,119 +5598,119 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="97">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="98">
   <autoFilter ref="A1:T3" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="96"/>
-    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="sourceStudyId" dataDxfId="95"/>
-    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="94"/>
-    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="93"/>
-    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="92"/>
-    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="91"/>
-    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="90"/>
-    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="89"/>
-    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="88"/>
-    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="87"/>
-    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="86"/>
-    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="85"/>
-    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="84"/>
-    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="83"/>
-    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="82"/>
-    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="81"/>
-    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="80"/>
-    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="79"/>
-    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="78"/>
-    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="77"/>
+    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="97"/>
+    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="sourceStudyId" dataDxfId="96"/>
+    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="95"/>
+    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="94"/>
+    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="93"/>
+    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="92"/>
+    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="91"/>
+    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="90"/>
+    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="89"/>
+    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="88"/>
+    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="87"/>
+    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="86"/>
+    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="85"/>
+    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="84"/>
+    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="83"/>
+    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="82"/>
+    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="81"/>
+    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="80"/>
+    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="79"/>
+    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="78"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="76" dataDxfId="75">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
   <autoFilter ref="A1:F2" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="74"/>
-    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="73"/>
-    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="72"/>
-    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="71"/>
-    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="70"/>
-    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="69"/>
+    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="75"/>
+    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="74"/>
+    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="73"/>
+    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="72"/>
+    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="71"/>
+    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="70"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="68" dataDxfId="67">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
   <autoFilter ref="A1:D2" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="66"/>
-    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="65"/>
-    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="64"/>
-    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="63"/>
+    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="67"/>
+    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="66"/>
+    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="65"/>
+    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="64"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="62" dataDxfId="61">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
   <autoFilter ref="A1:X2" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="60"/>
-    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="59"/>
-    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="58"/>
-    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="57"/>
-    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="56"/>
-    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="55"/>
-    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="53"/>
-    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="52"/>
-    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="51"/>
-    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="50"/>
-    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="49"/>
-    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="48"/>
-    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="47"/>
-    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="46"/>
-    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="45"/>
-    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="44"/>
-    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="43"/>
-    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="42"/>
-    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="41"/>
-    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="40"/>
-    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="39"/>
-    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="38"/>
-    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="37"/>
+    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="61"/>
+    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="60"/>
+    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="59"/>
+    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="58"/>
+    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="57"/>
+    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="56"/>
+    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="55"/>
+    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="54"/>
+    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="53"/>
+    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="52"/>
+    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="51"/>
+    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="50"/>
+    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="49"/>
+    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="48"/>
+    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="47"/>
+    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="46"/>
+    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="45"/>
+    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="44"/>
+    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="43"/>
+    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="42"/>
+    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="41"/>
+    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="40"/>
+    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="39"/>
+    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="38"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="37">
   <autoFilter ref="A1:C2" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="33"/>
+    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="34"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="32">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="33">
   <autoFilter ref="A1:F2" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="31"/>
-    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="30"/>
-    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="29">
+    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="31"/>
+    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="30">
       <calculatedColumnFormula>CONCATENATE(experimentalFactor[studyId],"-",experimentalFactor[expeFactorCode])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="29"/>
+    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="28"/>
+    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="27"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5709,16 +5733,16 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:G2" totalsRowShown="0" dataDxfId="25">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:G2" totalsRowShown="0" dataDxfId="26">
   <autoFilter ref="A1:G2" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="24"/>
-    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="23"/>
-    <tableColumn id="7" xr3:uid="{59210F7A-BDE1-4221-BA01-D09327E85900}" name="expeFactorLevelId" dataDxfId="0"/>
-    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="22"/>
-    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="21"/>
-    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="20"/>
-    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="25"/>
+    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{59210F7A-BDE1-4221-BA01-D09327E85900}" name="expeFactorLevelId" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="23"/>
+    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="22"/>
+    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="21"/>
+    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -11409,15 +11433,14 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:M997"/>
+  <dimension ref="A1:N997"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="7" width="20.42578125" customWidth="1"/>
-    <col min="8" max="13" width="10.5703125" customWidth="1"/>
-    <col min="16384" max="16384" width="11.42578125" customWidth="1"/>
+    <col min="1" max="8" width="20.42578125" customWidth="1"/>
+    <col min="9" max="14" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="36" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" s="36" customFormat="1" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="52" t="s">
         <v>66</v>
       </c>
@@ -11427,41 +11450,45 @@
       <c r="C1" s="52" t="s">
         <v>299</v>
       </c>
-      <c r="D1" s="52" t="s">
+      <c r="D1" s="66" t="s">
+        <v>702</v>
+      </c>
+      <c r="E1" s="52" t="s">
         <v>323</v>
       </c>
-      <c r="E1" s="53" t="s">
+      <c r="F1" s="53" t="s">
         <v>324</v>
       </c>
-      <c r="F1" s="51" t="s">
+      <c r="G1" s="51" t="s">
         <v>325</v>
       </c>
-      <c r="G1" s="51" t="s">
+      <c r="H1" s="51" t="s">
         <v>326</v>
       </c>
-      <c r="H1" s="41"/>
       <c r="I1" s="41"/>
       <c r="J1" s="41"/>
       <c r="K1" s="41"/>
       <c r="L1" s="41"/>
       <c r="M1" s="41"/>
-    </row>
-    <row r="2" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N1" s="41"/>
+    </row>
+    <row r="2" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="30"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="13"/>
+      <c r="D2" s="13"/>
+      <c r="E2" s="30"/>
       <c r="F2" s="13"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="43"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="30"/>
       <c r="I2" s="43"/>
       <c r="J2" s="43"/>
       <c r="K2" s="43"/>
       <c r="L2" s="43"/>
       <c r="M2" s="43"/>
-    </row>
-    <row r="3" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N2" s="43"/>
+    </row>
+    <row r="3" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -11469,14 +11496,15 @@
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
-      <c r="H3" s="43"/>
+      <c r="H3" s="7"/>
       <c r="I3" s="43"/>
       <c r="J3" s="43"/>
       <c r="K3" s="43"/>
       <c r="L3" s="43"/>
       <c r="M3" s="43"/>
-    </row>
-    <row r="4" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N3" s="43"/>
+    </row>
+    <row r="4" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
@@ -11484,14 +11512,15 @@
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
       <c r="G4" s="7"/>
-      <c r="H4" s="43"/>
+      <c r="H4" s="7"/>
       <c r="I4" s="43"/>
       <c r="J4" s="43"/>
       <c r="K4" s="43"/>
       <c r="L4" s="43"/>
       <c r="M4" s="43"/>
-    </row>
-    <row r="5" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N4" s="43"/>
+    </row>
+    <row r="5" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
@@ -11499,14 +11528,15 @@
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
       <c r="G5" s="7"/>
-      <c r="H5" s="43"/>
+      <c r="H5" s="7"/>
       <c r="I5" s="43"/>
       <c r="J5" s="43"/>
       <c r="K5" s="43"/>
       <c r="L5" s="43"/>
       <c r="M5" s="43"/>
-    </row>
-    <row r="6" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N5" s="43"/>
+    </row>
+    <row r="6" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
@@ -11514,14 +11544,15 @@
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
       <c r="G6" s="7"/>
-      <c r="H6" s="43"/>
+      <c r="H6" s="7"/>
       <c r="I6" s="43"/>
       <c r="J6" s="43"/>
       <c r="K6" s="43"/>
       <c r="L6" s="43"/>
       <c r="M6" s="43"/>
-    </row>
-    <row r="7" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N6" s="43"/>
+    </row>
+    <row r="7" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
@@ -11529,14 +11560,15 @@
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
       <c r="G7" s="7"/>
-      <c r="H7" s="43"/>
+      <c r="H7" s="7"/>
       <c r="I7" s="43"/>
       <c r="J7" s="43"/>
       <c r="K7" s="43"/>
       <c r="L7" s="43"/>
       <c r="M7" s="43"/>
-    </row>
-    <row r="8" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N7" s="43"/>
+    </row>
+    <row r="8" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
@@ -11544,14 +11576,15 @@
       <c r="E8" s="7"/>
       <c r="F8" s="7"/>
       <c r="G8" s="7"/>
-      <c r="H8" s="43"/>
+      <c r="H8" s="7"/>
       <c r="I8" s="43"/>
       <c r="J8" s="43"/>
       <c r="K8" s="43"/>
       <c r="L8" s="43"/>
       <c r="M8" s="43"/>
-    </row>
-    <row r="9" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="N8" s="43"/>
+    </row>
+    <row r="9" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="43"/>
       <c r="B9" s="43"/>
       <c r="C9" s="43"/>
@@ -11565,14 +11598,15 @@
       <c r="K9" s="43"/>
       <c r="L9" s="43"/>
       <c r="M9" s="43"/>
-    </row>
-    <row r="10" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="N9" s="43"/>
+    </row>
+    <row r="10" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -12555,9 +12589,12 @@
     <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2" xr:uid="{C9CAF3F9-1E81-44B5-A4D0-E0C67AD055FB}">
       <formula1>INDIRECT("study[studyId]")</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2" xr:uid="{65F4BB92-CA74-4B3B-B3E4-AF805E1DE54A}">
+      <formula1>INDIRECT("observationUnit[obsUnitId]")</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Added dataFileType to data file
This may be useful for categorising datasets and facilitating processing of common data files.
</commit_message>
<xml_diff>
--- a/Templates/MIAPPE_Spreadsheet_Template.xlsx
+++ b/Templates/MIAPPE_Spreadsheet_Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\MIAPPE\Templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D6E3BB-274C-4AD8-8440-6EF7D8E42893}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708EF98F-A854-4F9C-BCC9-F878A55FB8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="891" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="703">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="704">
   <si>
     <t>README</t>
   </si>
@@ -2345,6 +2345,9 @@
   </si>
   <si>
     <t>sourceObsUnitId</t>
+  </si>
+  <si>
+    <t>dataFileType</t>
   </si>
 </sst>
 </file>
@@ -2784,7 +2787,27 @@
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="140">
+  <dxfs count="141">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -5483,15 +5506,15 @@
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="MiappeStyle" pivot="0" count="9" xr9:uid="{59C54380-D204-4007-9CC6-0890CCDEE3C9}">
-      <tableStyleElement type="wholeTable" dxfId="139"/>
-      <tableStyleElement type="headerRow" dxfId="138"/>
-      <tableStyleElement type="totalRow" dxfId="137"/>
-      <tableStyleElement type="firstColumn" dxfId="136"/>
-      <tableStyleElement type="lastColumn" dxfId="135"/>
-      <tableStyleElement type="firstRowStripe" dxfId="134"/>
-      <tableStyleElement type="secondRowStripe" dxfId="133"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="132"/>
-      <tableStyleElement type="secondColumnStripe" dxfId="131"/>
+      <tableStyleElement type="wholeTable" dxfId="140"/>
+      <tableStyleElement type="headerRow" dxfId="139"/>
+      <tableStyleElement type="totalRow" dxfId="138"/>
+      <tableStyleElement type="firstColumn" dxfId="137"/>
+      <tableStyleElement type="lastColumn" dxfId="136"/>
+      <tableStyleElement type="firstRowStripe" dxfId="135"/>
+      <tableStyleElement type="secondRowStripe" dxfId="134"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="133"/>
+      <tableStyleElement type="secondColumnStripe" dxfId="132"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -5506,87 +5529,87 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="108" dataDxfId="107">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}" name="investigation" displayName="investigation" ref="A1:H2" totalsRowShown="0" headerRowDxfId="109" dataDxfId="108">
   <autoFilter ref="A1:H2" xr:uid="{D8AF6C71-E30B-48EC-A84C-21302F8FBBD8}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="106"/>
-    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="105"/>
-    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="104"/>
-    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="103"/>
-    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="102"/>
-    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="101"/>
-    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="100"/>
-    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="99"/>
+    <tableColumn id="1" xr3:uid="{25F01F79-3E24-44AF-B5E3-4EB20FD9A360}" name="investigationId" dataDxfId="107"/>
+    <tableColumn id="2" xr3:uid="{16E59F0F-AC6D-4504-A428-E7D7AC601401}" name="investigationTitle" dataDxfId="106"/>
+    <tableColumn id="3" xr3:uid="{4668A34F-CEFF-43A7-84AA-B014E3A90F47}" name="investigationDescription" dataDxfId="105"/>
+    <tableColumn id="4" xr3:uid="{403353FA-EBA5-418F-8273-81472CDF29D4}" name="submissionDate" dataDxfId="104"/>
+    <tableColumn id="5" xr3:uid="{18E43DB3-511F-4E0E-B357-B4A6E40F0660}" name="publicReleaseDate" dataDxfId="103"/>
+    <tableColumn id="6" xr3:uid="{91C01C8C-69AF-4B74-BA16-1C962EDAF32D}" name="license" dataDxfId="102"/>
+    <tableColumn id="7" xr3:uid="{E94BB99A-781A-4442-AD9C-7E4D99028DC9}" name="miappeVersion" dataDxfId="101"/>
+    <tableColumn id="8" xr3:uid="{91B9E445-65BD-412A-95C1-EA371F946FCA}" name="associatedPublication" dataDxfId="100"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table10.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:H2" insertRow="1" totalsRowShown="0" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}" name="observationUnit" displayName="observationUnit" ref="A1:H2" insertRow="1" totalsRowShown="0" dataDxfId="20">
   <autoFilter ref="A1:H2" xr:uid="{9A4F6851-A82A-4719-850B-9015CB0F68F5}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="16"/>
-    <tableColumn id="8" xr3:uid="{F4D9572F-C227-480C-812D-9943C387240C}" name="sourceObsUnitId" dataDxfId="0"/>
-    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="15"/>
-    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="14"/>
-    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="13"/>
-    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{67885524-1B5C-4054-BDDA-7439D87C65A3}" name="studyId" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{BD42E68A-B0EE-4F6E-9323-7BF9B4395F28}" name="biologicalMaterialId" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{ADEBC7D5-74AA-4299-BAA7-2B546D4FD4E2}" name="obsUnitId" dataDxfId="17"/>
+    <tableColumn id="8" xr3:uid="{F4D9572F-C227-480C-812D-9943C387240C}" name="sourceObsUnitId" dataDxfId="1"/>
+    <tableColumn id="4" xr3:uid="{9981E5B4-9802-41A5-B134-7A7924A4B125}" name="obsUnitType" dataDxfId="16"/>
+    <tableColumn id="5" xr3:uid="{CB30098B-ECC6-437C-9C2E-46BB51031C94}" name="externalId" dataDxfId="15"/>
+    <tableColumn id="6" xr3:uid="{B9F1BB11-5258-49AF-A8C5-372071AA9FF3}" name="spatialDistribution" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{7E1C2129-988B-4857-85FE-0F1EA951EBC7}" name="obsUnitFactorValue" dataDxfId="13"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table11.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="11" dataDxfId="10">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}" name="sample" displayName="sample" ref="A1:G2" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
   <autoFilter ref="A1:G2" xr:uid="{6D61A835-4FD1-495E-A537-D0167D8A5442}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="9"/>
-    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="8"/>
-    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="7"/>
-    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="6"/>
-    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="5"/>
-    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="4"/>
-    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{92A1E618-2F85-46E4-B7EF-76ED045C215B}" name="obsUnitId" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{A0DFEC37-340B-4DF8-907B-A9769602FD28}" name="sampleId" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{D455AF29-BE41-4DDA-A9B2-A46F4EEA6767}" name="developmentStage" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{C24109D3-E8A6-4810-A0A6-ACD6730F0D08}" name="anatomicalEntity" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{5C630D57-B424-4325-BC0C-BEEBEDC89DBB}" name="sampleDesc" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{CDEC6C64-2387-4FCF-9A2C-63F54020D0A0}" name="collectionDate" dataDxfId="5"/>
+    <tableColumn id="7" xr3:uid="{FFB2A4F7-3C7D-4BC5-AD9E-C14C20349305}" name="externalId" dataDxfId="4"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:U2" insertRow="1" totalsRowShown="0" dataDxfId="130">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="11" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}" name="observedVariable" displayName="observedVariable" ref="A1:U2" insertRow="1" totalsRowShown="0" dataDxfId="131">
   <autoFilter ref="A1:U2" xr:uid="{0EDFDBC4-F33A-4222-BE29-11AF54DCA710}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="129"/>
-    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="128"/>
-    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="127"/>
-    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="126"/>
-    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="125"/>
-    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="124"/>
-    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="123"/>
-    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="122"/>
-    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="121"/>
-    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="120"/>
-    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="119"/>
-    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="118"/>
-    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="117"/>
-    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="116"/>
-    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="115"/>
-    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="114"/>
-    <tableColumn id="19" xr3:uid="{EE91A801-8376-4314-ADFB-6E32C3AE8AE4}" name="timeScale" dataDxfId="113"/>
-    <tableColumn id="22" xr3:uid="{A52D8785-E3B2-4548-AA8A-0964285F0DB9}" name="participant" dataDxfId="112"/>
-    <tableColumn id="21" xr3:uid="{CA21FA4C-5A61-4852-9BA7-6FDDF22D4ADC}" name="participantAccession" dataDxfId="111"/>
-    <tableColumn id="20" xr3:uid="{3DF54E16-A553-4C7E-9762-C6517F5AD994}" name="participantRole" dataDxfId="110"/>
-    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="participantRoleAccession" dataDxfId="109"/>
+    <tableColumn id="1" xr3:uid="{52AF96AA-DC3C-4AE1-9B73-089CA835EB6D}" name="studyId" dataDxfId="130"/>
+    <tableColumn id="2" xr3:uid="{6323306B-E13C-4F7B-86EE-23DC8D1F262D}" name="variableId" dataDxfId="129"/>
+    <tableColumn id="3" xr3:uid="{DAD62536-0510-4DD9-9444-8EBA12087E02}" name="variableName" dataDxfId="128"/>
+    <tableColumn id="4" xr3:uid="{FD87E241-A1C6-4BF6-81FC-38FE779F31D6}" name="variableAccession" dataDxfId="127"/>
+    <tableColumn id="5" xr3:uid="{ED4E4010-EAC9-4FB0-9577-906D949DB6BF}" name="traitName" dataDxfId="126"/>
+    <tableColumn id="6" xr3:uid="{DA4A34B4-67B2-4ABC-9FA6-0EBFB54B964D}" name="traitEntity" dataDxfId="125"/>
+    <tableColumn id="7" xr3:uid="{9A164C4C-E33C-4F52-9CA0-56F6EC009A34}" name="traitEntityAccession" dataDxfId="124"/>
+    <tableColumn id="8" xr3:uid="{FB4A5310-40B1-46EF-B98F-2CA2AC87CE59}" name="traitCharacteristic" dataDxfId="123"/>
+    <tableColumn id="9" xr3:uid="{59E17836-2938-469A-A999-F34CBAA00B67}" name="traitCharacteristicAccession" dataDxfId="122"/>
+    <tableColumn id="10" xr3:uid="{7F9E3661-278E-45F4-A718-37C7F238C752}" name="traitAccession" dataDxfId="121"/>
+    <tableColumn id="11" xr3:uid="{F49AEE2B-9512-4C72-A2BF-C945026C81A0}" name="methodName" dataDxfId="120"/>
+    <tableColumn id="12" xr3:uid="{8099D3A2-60AE-4466-B82A-EEC20FC58B7B}" name="methodAccession" dataDxfId="119"/>
+    <tableColumn id="13" xr3:uid="{6291B064-7EBD-42CC-B89D-568748A16FA5}" name="methodDesc" dataDxfId="118"/>
+    <tableColumn id="14" xr3:uid="{A01FDF2D-88FC-405F-BF1E-14B20EABB5B5}" name="methodRef" dataDxfId="117"/>
+    <tableColumn id="15" xr3:uid="{A15211C8-293C-4DE6-87B9-CF94F470AE75}" name="scaleName" dataDxfId="116"/>
+    <tableColumn id="16" xr3:uid="{648CBC04-7A14-4F7F-A7AF-D119B1714850}" name="scaleAccession" dataDxfId="115"/>
+    <tableColumn id="19" xr3:uid="{EE91A801-8376-4314-ADFB-6E32C3AE8AE4}" name="timeScale" dataDxfId="114"/>
+    <tableColumn id="22" xr3:uid="{A52D8785-E3B2-4548-AA8A-0964285F0DB9}" name="participant" dataDxfId="113"/>
+    <tableColumn id="21" xr3:uid="{CA21FA4C-5A61-4852-9BA7-6FDDF22D4ADC}" name="participantAccession" dataDxfId="112"/>
+    <tableColumn id="20" xr3:uid="{3DF54E16-A553-4C7E-9762-C6517F5AD994}" name="participantRole" dataDxfId="111"/>
+    <tableColumn id="17" xr3:uid="{AD46E78F-5D35-4B20-9822-0B2F83C5680D}" name="participantRoleAccession" dataDxfId="110"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="2">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}" name="environmentParameters" displayName="environmentParameters" ref="A1:C3" totalsRowShown="0" headerRowDxfId="3">
   <autoFilter ref="A1:C3" xr:uid="{AB1F2FD5-EB26-42FD-AA78-B5395A6174BE}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{5E761B2A-3F92-4181-AF5D-F423F0564A09}" name="envParam"/>
@@ -5598,119 +5621,120 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="98">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}" name="study" displayName="study" ref="A1:T3" totalsRowShown="0" dataDxfId="99">
   <autoFilter ref="A1:T3" xr:uid="{5E227E83-2F05-4244-925F-48F9556390CD}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="97"/>
-    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="sourceStudyId" dataDxfId="96"/>
-    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="95"/>
-    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="94"/>
-    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="93"/>
-    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="92"/>
-    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="91"/>
-    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="90"/>
-    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="89"/>
-    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="88"/>
-    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="87"/>
-    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="86"/>
-    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="85"/>
-    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="84"/>
-    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="83"/>
-    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="82"/>
-    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="81"/>
-    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="80"/>
-    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="79"/>
-    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="78"/>
+    <tableColumn id="1" xr3:uid="{EE95CF2F-813E-4690-97C4-79C304F65B9C}" name="studyId" dataDxfId="98"/>
+    <tableColumn id="20" xr3:uid="{B540CC62-E9C4-45D9-ADBE-8B9EAB4D0769}" name="sourceStudyId" dataDxfId="97"/>
+    <tableColumn id="2" xr3:uid="{799EAD4E-60F7-47E4-B3B2-8BD859F0673D}" name="studyTitle" dataDxfId="96"/>
+    <tableColumn id="3" xr3:uid="{A2063A94-CC8E-425D-A71D-C0EDE3148180}" name="studyDescription" dataDxfId="95"/>
+    <tableColumn id="4" xr3:uid="{4DCF1664-298B-4E1C-8B80-483A31FB0BDB}" name="studyStartDate" dataDxfId="94"/>
+    <tableColumn id="5" xr3:uid="{E557DB42-3379-4598-AAF9-21798BC64DAB}" name="studyEndDate" dataDxfId="93"/>
+    <tableColumn id="6" xr3:uid="{1EEA2EC5-CA19-40B4-9DFB-2DE9A9E916EA}" name="contactInst" dataDxfId="92"/>
+    <tableColumn id="7" xr3:uid="{E0A5C222-CFE5-4E9C-8E84-0892043DBD21}" name="locationCountry" dataDxfId="91"/>
+    <tableColumn id="8" xr3:uid="{7B635D2A-56C5-48B0-A880-E33ADE030AB1}" name="siteName" dataDxfId="90"/>
+    <tableColumn id="9" xr3:uid="{2F8227C3-F11C-4DAA-93EB-CEBD94FF81A9}" name="locationLatitude" dataDxfId="89"/>
+    <tableColumn id="10" xr3:uid="{6A14EB46-0BF4-45C6-9048-E1B7D13E633A}" name="locationLongitude" dataDxfId="88"/>
+    <tableColumn id="11" xr3:uid="{9954429A-AA41-408C-BB04-D73EDB89D73F}" name="locationAltitude" dataDxfId="87"/>
+    <tableColumn id="12" xr3:uid="{39FEDA43-D994-4742-B319-3DFED43EF79B}" name="expeDesignDesc" dataDxfId="86"/>
+    <tableColumn id="13" xr3:uid="{C9F6A881-1CF1-4AD9-8305-B7E26FD78E3B}" name="expeDesignType" dataDxfId="85"/>
+    <tableColumn id="14" xr3:uid="{253A58C7-1A2A-4D25-9622-3AE33F89A685}" name="obsUnitLevelHierarchy" dataDxfId="84"/>
+    <tableColumn id="15" xr3:uid="{10DCEB5F-0BF5-4476-83E5-B973A516A8CD}" name="obsUnitDesc" dataDxfId="83"/>
+    <tableColumn id="16" xr3:uid="{0D36E7FE-2245-4B79-9A59-4C64590731A5}" name="growthFacilityDesc" dataDxfId="82"/>
+    <tableColumn id="17" xr3:uid="{599307E8-6E88-4D3F-BF48-ADF70D109D18}" name="growthFacilityType" dataDxfId="81"/>
+    <tableColumn id="18" xr3:uid="{63403E81-283C-4E2E-984D-9EFC0886E90C}" name="culturalPractice" dataDxfId="80"/>
+    <tableColumn id="19" xr3:uid="{E74D4B3A-67BC-482F-8485-FC7D9088A8B6}" name="expeDesignMap" dataDxfId="79"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="77" dataDxfId="76">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}" name="person" displayName="person" ref="A1:F2" insertRow="1" totalsRowShown="0" headerRowDxfId="78" dataDxfId="77">
   <autoFilter ref="A1:F2" xr:uid="{2FBCF0B0-7AB0-436F-9431-67BEDDE78EB3}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="75"/>
-    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="74"/>
-    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="73"/>
-    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="72"/>
-    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="71"/>
-    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="70"/>
+    <tableColumn id="1" xr3:uid="{49A703DB-336A-4F60-9DA6-8249763A2765}" name="studyId" dataDxfId="76"/>
+    <tableColumn id="2" xr3:uid="{65039BF4-A122-4B88-8EB2-FD3ED61B8912}" name="personName" dataDxfId="75"/>
+    <tableColumn id="3" xr3:uid="{4B7588A4-B756-4E28-B8A4-AFB8D62031B4}" name="personEmail" dataDxfId="74"/>
+    <tableColumn id="4" xr3:uid="{639FC837-B543-4A62-B2C2-3EE761EF5EF7}" name="personId" dataDxfId="73"/>
+    <tableColumn id="5" xr3:uid="{593F31A8-CDAA-47CF-89F3-2902C6B8D3C8}" name="personRole" dataDxfId="72"/>
+    <tableColumn id="6" xr3:uid="{5FCF059F-31D5-4218-8D81-DC379C42EAF4}" name="personAffiliation" dataDxfId="71"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:D2" insertRow="1" totalsRowShown="0" headerRowDxfId="69" dataDxfId="68">
-  <autoFilter ref="A1:D2" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}"/>
-  <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="67"/>
-    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="66"/>
-    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="65"/>
-    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="64"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}" name="dataFile" displayName="dataFile" ref="A1:E2" insertRow="1" totalsRowShown="0" headerRowDxfId="70" dataDxfId="69">
+  <autoFilter ref="A1:E2" xr:uid="{6A3BD8AE-973B-42AE-B791-86C37DE5452E}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{AD6A7B95-2E4C-4264-86B4-35031C8932E3}" name="studyId" dataDxfId="68"/>
+    <tableColumn id="2" xr3:uid="{A5C92CF7-B78F-4910-A250-8A16D6E7889C}" name="dataFileLink" dataDxfId="67"/>
+    <tableColumn id="3" xr3:uid="{620AC217-74DA-496A-9696-16EF7D98E86C}" name="dataFileDesc" dataDxfId="66"/>
+    <tableColumn id="5" xr3:uid="{AFC6BCDB-79B5-4940-A3BB-0EEC9F1306A5}" name="dataFileType" dataDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{79F128D7-FDA0-4F62-B04B-DAEE7E495850}" name="dataFileVersion" dataDxfId="65"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="63" dataDxfId="62">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}" name="biologicalMaterial" displayName="biologicalMaterial" ref="A1:X2" insertRow="1" totalsRowShown="0" headerRowDxfId="64" dataDxfId="63">
   <autoFilter ref="A1:X2" xr:uid="{CD8645E7-2CD1-4841-84CC-19654A603435}"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="61"/>
-    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="60"/>
-    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="59"/>
-    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="58"/>
-    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="57"/>
-    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="56"/>
-    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="55"/>
-    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="54"/>
-    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="53"/>
-    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="52"/>
-    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="51"/>
-    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="50"/>
-    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="49"/>
-    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="48"/>
-    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="47"/>
-    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="46"/>
-    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="45"/>
-    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="44"/>
-    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="43"/>
-    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="42"/>
-    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="41"/>
-    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="40"/>
-    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="39"/>
-    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="38"/>
+    <tableColumn id="1" xr3:uid="{71E6992E-3AF7-4C8A-9C1E-930C105005E2}" name="studyId" dataDxfId="62"/>
+    <tableColumn id="2" xr3:uid="{BA8B45A2-9F79-4EE6-A38F-EF56D5CE4A1A}" name="biologicalMaterialId" dataDxfId="61"/>
+    <tableColumn id="3" xr3:uid="{546FEA19-FA9D-47D3-BF6E-57CDA029B0A3}" name="biologicalMaterialExtId" dataDxfId="60"/>
+    <tableColumn id="4" xr3:uid="{0DD21880-A5E2-4076-AA9F-554DE7C7E0D1}" name="organism" dataDxfId="59"/>
+    <tableColumn id="5" xr3:uid="{9760C8F1-7162-4A84-80C2-FBEC779AFAD0}" name="genus" dataDxfId="58"/>
+    <tableColumn id="6" xr3:uid="{D7026284-DE40-4B04-A583-983A0B5FB5BB}" name="species" dataDxfId="57"/>
+    <tableColumn id="7" xr3:uid="{22046373-BBD5-4919-AC4C-AA8E91D97026}" name="infraspecificName" dataDxfId="56"/>
+    <tableColumn id="8" xr3:uid="{579B0DCA-BD9C-4E7B-BB3B-3FB19A4CBCA3}" name="biologicalMaterialLatitude" dataDxfId="55"/>
+    <tableColumn id="9" xr3:uid="{A7E064AC-CDCF-4898-BEF3-07CF88887A4E}" name="biologicalMaterialLongitude" dataDxfId="54"/>
+    <tableColumn id="10" xr3:uid="{D55DD07C-0BE6-4D7D-80E1-B7195245711A}" name="biologicalMaterialAltitude" dataDxfId="53"/>
+    <tableColumn id="11" xr3:uid="{CA82A017-8E46-417C-9A1F-D7010C7B489F}" name="biologicalMaterialCoordUncertainty" dataDxfId="52"/>
+    <tableColumn id="12" xr3:uid="{16F6B082-1241-4094-AFDC-6E6F5B63F502}" name="biologicalMaterialPreprocessing" dataDxfId="51"/>
+    <tableColumn id="13" xr3:uid="{16F5564F-9F1B-4CEB-8DEC-4F46E89C2EB5}" name="materialSourceId" dataDxfId="50"/>
+    <tableColumn id="14" xr3:uid="{0AB5DA63-1709-41B8-9FAD-5B1A8A45E649}" name="materialSourceDoi" dataDxfId="49"/>
+    <tableColumn id="15" xr3:uid="{26116E4A-CA0A-4D6C-A863-AEA24B0E0C24}" name="materialSourceAccNumber" dataDxfId="48"/>
+    <tableColumn id="16" xr3:uid="{0C2E647E-5127-470F-859E-ED727EEFA3B9}" name="materialSourceAccName" dataDxfId="47"/>
+    <tableColumn id="17" xr3:uid="{B6097563-29EF-4C10-9096-04A2C164B15A}" name="materialSourceInstCode" dataDxfId="46"/>
+    <tableColumn id="18" xr3:uid="{BEA38246-EAA3-4450-B29F-D608607C2513}" name="materialSourceInstName" dataDxfId="45"/>
+    <tableColumn id="19" xr3:uid="{E8257013-CD5D-4534-9CD0-08D9EBBE7EF0}" name="materialSourceOtherIds" dataDxfId="44"/>
+    <tableColumn id="20" xr3:uid="{BE0E6D94-2ED0-4863-9DE5-9AA6BD4643D6}" name="materialSourceLatitude" dataDxfId="43"/>
+    <tableColumn id="21" xr3:uid="{BD849876-C99C-4475-87D4-DEECBE575F67}" name="materialSourceLongitude" dataDxfId="42"/>
+    <tableColumn id="22" xr3:uid="{0C871681-B897-43DD-A6BE-F03CAA6574F6}" name="materialSourceAltitude" dataDxfId="41"/>
+    <tableColumn id="23" xr3:uid="{ECC67BD8-3E1F-4A97-95B0-A9CCE07839CA}" name="materialSourceCoordUncertainty" dataDxfId="40"/>
+    <tableColumn id="24" xr3:uid="{C66E78D2-DB97-4D59-8D52-ECE79ED6BB86}" name="materialSourceDesc" dataDxfId="39"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="37">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}" name="environment" displayName="environment" ref="A1:C2" insertRow="1" totalsRowShown="0" headerRowDxfId="38">
   <autoFilter ref="A1:C2" xr:uid="{1C4F81EC-6E53-43AA-B6CF-9BA631481909}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="36"/>
-    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="35"/>
-    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="34"/>
+    <tableColumn id="1" xr3:uid="{08C0BD82-D970-44E6-99E3-B4872FECEFE5}" name="studyId" dataDxfId="37"/>
+    <tableColumn id="2" xr3:uid="{F9DC7CC5-88B3-4A9A-B462-9FB971836B81}" name="envParam" dataDxfId="36"/>
+    <tableColumn id="3" xr3:uid="{65E72A00-3C03-4A17-922C-EE6A4A3D8D80}" name="envParamValue" dataDxfId="35"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="33">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}" name="experimentalFactor" displayName="experimentalFactor" ref="A1:F2" totalsRowShown="0" headerRowDxfId="34">
   <autoFilter ref="A1:F2" xr:uid="{9DB56221-E63F-405B-979B-FD6B29D3B9AE}"/>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="31"/>
-    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="30">
+    <tableColumn id="1" xr3:uid="{8033D24B-35FE-4753-9513-1BA7E8E27122}" name="studyId" dataDxfId="33"/>
+    <tableColumn id="6" xr3:uid="{8AF0BF35-BAC4-4E9A-A1CC-B83DC7399496}" name="expeFactorCode" dataDxfId="32"/>
+    <tableColumn id="5" xr3:uid="{67BFB12E-F4AF-4C45-B7B6-4791A656C30A}" name="expeFactorId" dataDxfId="31">
       <calculatedColumnFormula>CONCATENATE(experimentalFactor[studyId],"-",experimentalFactor[expeFactorCode])</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{0E59C639-24C1-40B6-85BF-F9DA37B289AF}" name="expeFactorType" dataDxfId="30"/>
+    <tableColumn id="3" xr3:uid="{45088180-C6C0-4340-B527-76C01394AC82}" name="expeFactorDesc" dataDxfId="29"/>
+    <tableColumn id="4" xr3:uid="{79953CF7-2E96-4871-AAED-69F19C77A395}" name="expeFactorValues" dataDxfId="28"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5733,16 +5757,16 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:G2" totalsRowShown="0" dataDxfId="26">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}" name="event" displayName="event" ref="A1:G2" totalsRowShown="0" dataDxfId="27">
   <autoFilter ref="A1:G2" xr:uid="{E52243D7-2662-4692-B203-793CCE48631D}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="25"/>
-    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{59210F7A-BDE1-4221-BA01-D09327E85900}" name="expeFactorLevelId" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="23"/>
-    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="22"/>
-    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="21"/>
-    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{DB25986C-BD6F-40F9-A226-C9A11BBDF460}" name="studyId" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{6EE72788-DEAD-4FC0-9383-C6415EC5E8A5}" name="obsUnitId" dataDxfId="25"/>
+    <tableColumn id="7" xr3:uid="{59210F7A-BDE1-4221-BA01-D09327E85900}" name="expeFactorLevelId" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{0DDCD5FF-AC45-4794-9B28-BBD982C1FB84}" name="eventType" dataDxfId="24"/>
+    <tableColumn id="4" xr3:uid="{F8E58477-EC1C-4F97-B99C-B939249E19E9}" name="eventAccNumber" dataDxfId="23"/>
+    <tableColumn id="5" xr3:uid="{E826B0E9-8F41-4E58-9D61-690A1F38823F}" name="eventDesc" dataDxfId="22"/>
+    <tableColumn id="6" xr3:uid="{6ABA4348-63AB-41DB-837E-5BE18C09264B}" name="eventDate" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="MiappeStyle" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -21906,15 +21930,14 @@
   <sheetPr>
     <tabColor rgb="FF008000"/>
   </sheetPr>
-  <dimension ref="A1:X997"/>
+  <dimension ref="A1:Y997"/>
   <sheetFormatPr defaultColWidth="14.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="4" width="20.42578125" customWidth="1"/>
-    <col min="16383" max="16383" width="11.42578125" customWidth="1"/>
-    <col min="16384" max="16384" width="11.5703125" customWidth="1"/>
+    <col min="1" max="5" width="20.42578125" customWidth="1"/>
+    <col min="16384" max="16384" width="11.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:25" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="52" t="s">
         <v>66</v>
       </c>
@@ -21925,9 +21948,11 @@
         <v>160</v>
       </c>
       <c r="D1" s="52" t="s">
+        <v>703</v>
+      </c>
+      <c r="E1" s="52" t="s">
         <v>161</v>
       </c>
-      <c r="E1" s="36"/>
       <c r="F1" s="36"/>
       <c r="G1" s="36"/>
       <c r="H1" s="36"/>
@@ -21947,57 +21972,65 @@
       <c r="V1" s="36"/>
       <c r="W1" s="36"/>
       <c r="X1" s="36"/>
-    </row>
-    <row r="2" spans="1:24" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="Y1" s="36"/>
+    </row>
+    <row r="2" spans="1:25" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="30"/>
       <c r="B2" s="13"/>
       <c r="C2" s="13"/>
       <c r="D2" s="13"/>
-    </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="E2" s="13"/>
+    </row>
+    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
       <c r="A3" s="7"/>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
       <c r="D3" s="7"/>
-    </row>
-    <row r="4" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E3" s="7"/>
+    </row>
+    <row r="4" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="7"/>
       <c r="C4" s="7"/>
       <c r="D4" s="7"/>
-    </row>
-    <row r="5" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" s="7"/>
+    </row>
+    <row r="5" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="7"/>
       <c r="C5" s="7"/>
       <c r="D5" s="7"/>
-    </row>
-    <row r="6" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="7"/>
+    </row>
+    <row r="6" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="7"/>
       <c r="D6" s="7"/>
-    </row>
-    <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E6" s="7"/>
+    </row>
+    <row r="7" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="7"/>
       <c r="C7" s="7"/>
       <c r="D7" s="7"/>
-    </row>
-    <row r="8" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E7" s="7"/>
+    </row>
+    <row r="8" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="7"/>
       <c r="C8" s="7"/>
       <c r="D8" s="7"/>
-    </row>
-    <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="E8" s="7"/>
+    </row>
+    <row r="9" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="11" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="1:25" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>